<commit_message>
feat: update forecasting data pipeline and integrate price estimation feature
- Changed input data source from Final_Data.xlsx to Data/v3/master_v3.csv, increasing listings from 3,037 to 6,703.
- Updated data processing script to normalize property types and legal statuses.
- Added price estimation endpoint to the API, allowing comparison of asking prices with ML estimates.
- Implemented price estimation logic in the backend, including validation against training domain constraints.
- Created frontend components to display price estimates and integrated them into property detail pages.
- Added unit tests for price estimation functionality and legal status normalization.
- Updated requirements to include necessary libraries for new features.
</commit_message>
<xml_diff>
--- a/price-prediction/model_evaluation.xlsx
+++ b/price-prediction/model_evaluation.xlsx
@@ -468,19 +468,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6942</v>
+        <v>0.748</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2886</v>
+        <v>0.2671</v>
       </c>
       <c r="D2" t="n">
-        <v>2.346</v>
+        <v>2.111</v>
       </c>
       <c r="E2" t="n">
-        <v>1.271</v>
+        <v>1.116</v>
       </c>
       <c r="F2" t="n">
-        <v>26.31</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="3">
@@ -490,19 +490,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7923</v>
+        <v>0.8321</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2378</v>
+        <v>0.218</v>
       </c>
       <c r="D3" t="n">
-        <v>1.736</v>
+        <v>1.508</v>
       </c>
       <c r="E3" t="n">
-        <v>0.856</v>
+        <v>0.712</v>
       </c>
       <c r="F3" t="n">
-        <v>19.98</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="4">
@@ -512,19 +512,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7971</v>
+        <v>0.833</v>
       </c>
       <c r="C4" t="n">
-        <v>0.235</v>
+        <v>0.2174</v>
       </c>
       <c r="D4" t="n">
-        <v>1.773</v>
+        <v>1.56</v>
       </c>
       <c r="E4" t="n">
-        <v>0.931</v>
+        <v>0.82</v>
       </c>
       <c r="F4" t="n">
-        <v>19.91</v>
+        <v>19.21</v>
       </c>
     </row>
   </sheetData>
@@ -595,22 +595,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>463</v>
+        <v>1002</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6942</v>
+        <v>0.748</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2886</v>
+        <v>0.2671</v>
       </c>
       <c r="F2" t="n">
-        <v>2.346</v>
+        <v>2.111</v>
       </c>
       <c r="G2" t="n">
-        <v>1.271</v>
+        <v>1.116</v>
       </c>
       <c r="H2" t="n">
-        <v>26.31</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>83</v>
+        <v>279</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5972</v>
+        <v>0.7478</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2664</v>
+        <v>0.2168</v>
       </c>
       <c r="F3" t="n">
-        <v>1.249</v>
+        <v>1.043</v>
       </c>
       <c r="G3" t="n">
-        <v>0.928</v>
+        <v>0.747</v>
       </c>
       <c r="H3" t="n">
-        <v>28.09</v>
+        <v>23.53</v>
       </c>
     </row>
     <row r="4">
@@ -655,22 +655,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>380</v>
+        <v>723</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6259</v>
+        <v>0.64</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2932</v>
+        <v>0.2841</v>
       </c>
       <c r="F4" t="n">
-        <v>2.586</v>
+        <v>2.523</v>
       </c>
       <c r="G4" t="n">
-        <v>1.402</v>
+        <v>1.347</v>
       </c>
       <c r="H4" t="n">
-        <v>25.92</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="5">
@@ -685,22 +685,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>463</v>
+        <v>1002</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7923</v>
+        <v>0.8321</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2378</v>
+        <v>0.218</v>
       </c>
       <c r="F5" t="n">
-        <v>1.736</v>
+        <v>1.508</v>
       </c>
       <c r="G5" t="n">
-        <v>0.856</v>
+        <v>0.712</v>
       </c>
       <c r="H5" t="n">
-        <v>19.98</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="6">
@@ -715,22 +715,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>83</v>
+        <v>279</v>
       </c>
       <c r="D6" t="n">
-        <v>0.802</v>
+        <v>0.89</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1867</v>
+        <v>0.1432</v>
       </c>
       <c r="F6" t="n">
-        <v>0.732</v>
+        <v>0.61</v>
       </c>
       <c r="G6" t="n">
-        <v>0.437</v>
+        <v>0.336</v>
       </c>
       <c r="H6" t="n">
-        <v>16.85</v>
+        <v>13.47</v>
       </c>
     </row>
     <row r="7">
@@ -745,22 +745,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>380</v>
+        <v>723</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7333</v>
+        <v>0.7416</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2476</v>
+        <v>0.2407</v>
       </c>
       <c r="F7" t="n">
-        <v>1.955</v>
+        <v>1.854</v>
       </c>
       <c r="G7" t="n">
-        <v>0.968</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>20.66</v>
+        <v>20.06</v>
       </c>
     </row>
     <row r="8">
@@ -775,22 +775,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>463</v>
+        <v>1002</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7971</v>
+        <v>0.833</v>
       </c>
       <c r="E8" t="n">
-        <v>0.235</v>
+        <v>0.2174</v>
       </c>
       <c r="F8" t="n">
-        <v>1.773</v>
+        <v>1.56</v>
       </c>
       <c r="G8" t="n">
-        <v>0.931</v>
+        <v>0.82</v>
       </c>
       <c r="H8" t="n">
-        <v>19.91</v>
+        <v>19.21</v>
       </c>
     </row>
     <row r="9">
@@ -805,22 +805,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>83</v>
+        <v>279</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8507</v>
+        <v>0.9005</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1622</v>
+        <v>0.1362</v>
       </c>
       <c r="F9" t="n">
-        <v>0.665</v>
+        <v>0.599</v>
       </c>
       <c r="G9" t="n">
-        <v>0.358</v>
+        <v>0.375</v>
       </c>
       <c r="H9" t="n">
-        <v>14.89</v>
+        <v>13.56</v>
       </c>
     </row>
     <row r="10">
@@ -835,22 +835,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>380</v>
+        <v>723</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7321</v>
+        <v>0.7398</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2481</v>
+        <v>0.2416</v>
       </c>
       <c r="F10" t="n">
-        <v>2.015</v>
+        <v>1.931</v>
       </c>
       <c r="G10" t="n">
-        <v>1.113</v>
+        <v>1.127</v>
       </c>
       <c r="H10" t="n">
-        <v>21.01</v>
+        <v>21.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>